<commit_message>
started titanic kaggle competion
</commit_message>
<xml_diff>
--- a/Temperature/country temp2.xlsx
+++ b/Temperature/country temp2.xlsx
@@ -425,10 +425,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>2020</t>
@@ -452,17 +457,14 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>1980</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>index</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>37.54069403</v>
@@ -479,15 +481,12 @@
       <c r="F2" t="n">
         <v>35.4778625</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Kazakhstan</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>38.8475843</v>
@@ -504,15 +503,12 @@
       <c r="F3" t="n">
         <v>35.214553</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Russia</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
       </c>
       <c r="B4" t="n">
         <v>37.02080352</v>
@@ -529,15 +525,12 @@
       <c r="F4" t="n">
         <v>35.74441246</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>37.2810333</v>
@@ -554,15 +547,12 @@
       <c r="F5" t="n">
         <v>36.0268047</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>36.79494851</v>
@@ -578,11 +568,6 @@
       </c>
       <c r="F6" t="n">
         <v>36.0974373</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>